<commit_message>
Classify all rows as service's own site vs comparison/roundup article
Add サイト種別 column: 自社サービス公式サイト (52), 自社サービス（URL不明） (11),
比較・まとめ記事（第三者サイト） (123). Used to target the retry batch at
own-service rows only, since comparison-article rows' 会社名/費用 fields
don't map to a single company.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SEO記事AI代行会社リスト.xlsx
+++ b/SEO記事AI代行会社リスト.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SEO記事AI代行会社" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEO記事AI代行会社" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:I188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -446,6 +446,7 @@
     <col width="35" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -496,6 +497,11 @@
           <t>費用</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>サイト種別</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -536,6 +542,11 @@
           <t>20,000円～（テスト発注可能、業界により変動）</t>
         </is>
       </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -576,6 +587,11 @@
           <t>最低5記事/月。具体的な金額は要問い合わせ</t>
         </is>
       </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -616,6 +632,11 @@
           <t>1本14,800円～</t>
         </is>
       </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -656,6 +677,11 @@
           <t>15,000円/記事～</t>
         </is>
       </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -696,6 +722,11 @@
           <t>1記事4,980円（税別）、月2～100記事対応</t>
         </is>
       </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -736,6 +767,11 @@
           <t>1記事18,000～20,000円（発注数により変動）</t>
         </is>
       </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -776,6 +812,11 @@
           <t>月額495円～29,700円（複数プラン展開）</t>
         </is>
       </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -816,6 +857,11 @@
           <t>要問い合わせ</t>
         </is>
       </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -856,6 +902,11 @@
           <t>1記事12,000円～</t>
         </is>
       </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -896,6 +947,11 @@
           <t>要問い合わせ</t>
         </is>
       </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -936,6 +992,11 @@
           <t>要問い合わせ</t>
         </is>
       </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -976,6 +1037,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1016,6 +1082,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1056,6 +1127,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1096,6 +1172,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1136,6 +1217,11 @@
           <t>4,800円〜（文字数・内容により変動）</t>
         </is>
       </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1176,6 +1262,11 @@
           <t>スタンダードプラン文字単価4円〜、AI記事代行プラン1本16,000円〜、通常プラン文字単価4.5円〜</t>
         </is>
       </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1216,6 +1307,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1256,6 +1352,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1296,6 +1397,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1336,6 +1442,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1376,6 +1487,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1416,6 +1532,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1456,6 +1577,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1496,6 +1622,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1536,6 +1667,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1576,6 +1712,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1616,6 +1757,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1656,6 +1802,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1696,6 +1847,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1736,6 +1892,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -1776,6 +1937,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1816,6 +1982,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -1856,6 +2027,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1896,6 +2072,11 @@
           <t>1記事9,000円〜</t>
         </is>
       </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -1936,6 +2117,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -1976,6 +2162,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2016,6 +2207,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2056,6 +2252,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2096,6 +2297,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2136,6 +2342,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -2176,6 +2387,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -2216,6 +2432,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -2256,6 +2477,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -2296,6 +2522,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -2336,6 +2567,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -2376,6 +2612,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -2416,6 +2657,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -2456,6 +2702,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -2496,6 +2747,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -2536,6 +2792,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -2576,6 +2837,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -2616,6 +2882,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -2656,6 +2927,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -2696,6 +2972,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -2736,6 +3017,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2776,6 +3062,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -2816,6 +3107,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -2856,6 +3152,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -2896,6 +3197,11 @@
           <t>1記事15,000円〜</t>
         </is>
       </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -2936,6 +3242,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -2976,6 +3287,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -3016,6 +3332,11 @@
           <t>20,000円〜（テスト発注可能、業界により変動）</t>
         </is>
       </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -3056,6 +3377,11 @@
           <t>最低5記事/月。具体的な金額は要問い合わせ</t>
         </is>
       </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -3096,6 +3422,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -3136,6 +3467,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -3176,6 +3512,11 @@
           <t>1本16,000円〜</t>
         </is>
       </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -3216,6 +3557,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -3256,6 +3602,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -3296,6 +3647,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -3336,6 +3692,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -3376,6 +3737,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -3416,6 +3782,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -3456,6 +3827,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス（URL不明）</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -3496,6 +3872,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -3536,6 +3917,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -3576,6 +3962,11 @@
           <t>20,000円〜（テスト発注可能、業界により変動）</t>
         </is>
       </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -3616,6 +4007,11 @@
           <t>最低5記事/月。具体的な金額は要問い合わせ</t>
         </is>
       </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -3656,6 +4052,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -3696,6 +4097,11 @@
           <t>15,000円/記事〜</t>
         </is>
       </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -3736,6 +4142,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -3776,6 +4187,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -3816,6 +4232,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
@@ -3856,6 +4277,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -3896,6 +4322,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
@@ -3936,6 +4367,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -3976,6 +4412,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -4016,6 +4457,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -4056,6 +4502,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
@@ -4096,6 +4547,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -4136,6 +4592,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
@@ -4176,6 +4637,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -4216,6 +4682,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
@@ -4256,6 +4727,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -4296,6 +4772,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -4336,6 +4817,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -4376,6 +4862,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -4416,6 +4907,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -4456,6 +4952,11 @@
           <t>文字単価2円〜（プランにより変動）</t>
         </is>
       </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -4496,6 +4997,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -4536,6 +5042,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
@@ -4576,6 +5087,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -4616,6 +5132,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
@@ -4656,6 +5177,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -4696,6 +5222,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
@@ -4736,6 +5267,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -4776,6 +5312,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -4816,6 +5357,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -4856,6 +5402,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
@@ -4896,6 +5447,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -4936,6 +5492,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
@@ -4976,6 +5537,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -5016,6 +5582,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
@@ -5056,6 +5627,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -5096,6 +5672,11 @@
           <t>月額5記事50,000円（税抜）等の定額プランあり</t>
         </is>
       </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
@@ -5136,6 +5717,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -5176,6 +5762,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
@@ -5216,6 +5807,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -5256,6 +5852,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -5296,6 +5897,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -5336,6 +5942,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
@@ -5376,6 +5987,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I124" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -5416,6 +6032,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -5456,6 +6077,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I126" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -5496,6 +6122,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
@@ -5536,6 +6167,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I128" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -5576,6 +6212,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
@@ -5616,6 +6257,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I130" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -5656,6 +6302,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I131" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
@@ -5696,6 +6347,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I132" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -5736,6 +6392,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
@@ -5776,6 +6437,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I134" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -5816,6 +6482,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I135" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
@@ -5856,6 +6527,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I136" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -5896,6 +6572,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
@@ -5936,6 +6617,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I138" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -5976,6 +6662,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I139" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
@@ -6016,6 +6707,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I140" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -6056,6 +6752,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I141" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
@@ -6096,6 +6797,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I142" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -6136,6 +6842,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I143" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
@@ -6176,6 +6887,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I144" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -6216,6 +6932,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I145" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
@@ -6256,6 +6977,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I146" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -6296,6 +7022,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I147" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
@@ -6336,6 +7067,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I148" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -6376,6 +7112,11 @@
           <t>3,000文字/記事 18,000円〜（パッケージにより変動）</t>
         </is>
       </c>
+      <c r="I149" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
@@ -6416,6 +7157,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -6456,6 +7202,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I151" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
@@ -6496,6 +7247,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -6536,6 +7292,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I153" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
@@ -6576,6 +7337,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I154" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
@@ -6616,6 +7382,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I155" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
@@ -6656,6 +7427,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I156" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -6696,6 +7472,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
@@ -6736,6 +7517,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
@@ -6776,6 +7562,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I159" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
@@ -6816,6 +7607,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I160" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
@@ -6856,6 +7652,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I161" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
@@ -6896,6 +7697,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I162" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
@@ -6936,6 +7742,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I163" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
@@ -6976,6 +7787,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I164" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -7016,6 +7832,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I165" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
@@ -7056,6 +7877,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I166" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -7096,6 +7922,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I167" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
@@ -7136,6 +7967,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I168" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
@@ -7176,6 +8012,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I169" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="3" t="inlineStr">
@@ -7216,6 +8057,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I170" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="inlineStr">
@@ -7256,6 +8102,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I171" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="3" t="inlineStr">
@@ -7296,6 +8147,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I172" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="inlineStr">
@@ -7336,6 +8192,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I173" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
@@ -7376,6 +8237,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="inlineStr">
@@ -7416,6 +8282,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I175" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="3" t="inlineStr">
@@ -7456,6 +8327,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I176" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="inlineStr">
@@ -7496,6 +8372,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I177" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="3" t="inlineStr">
@@ -7536,6 +8417,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I178" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="inlineStr">
@@ -7576,6 +8462,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I179" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="3" t="inlineStr">
@@ -7616,6 +8507,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I180" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="inlineStr">
@@ -7656,6 +8552,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I181" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="3" t="inlineStr">
@@ -7696,6 +8597,11 @@
           <t>無料</t>
         </is>
       </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
+          <t>自社サービス公式サイト</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">
@@ -7736,6 +8642,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I183" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="3" t="inlineStr">
@@ -7776,6 +8687,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I184" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="inlineStr">
@@ -7816,6 +8732,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I185" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="3" t="inlineStr">
@@ -7856,6 +8777,11 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="inlineStr">
@@ -7896,6 +8822,11 @@
           <t>月額3万円〜10万円前後で一定本数のコンテンツを依頼できるパックプランあり</t>
         </is>
       </c>
+      <c r="I187" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="3" t="inlineStr">
@@ -7936,10 +8867,15 @@
           <t>取得不可</t>
         </is>
       </c>
+      <c r="I188" s="3" t="inlineStr">
+        <is>
+          <t>比較・まとめ記事（第三者サイト）</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>